<commit_message>
Committing changes before moving to Git
git-svn-id: https://svn2.phy.bris.ac.uk/svn/uob-hep-pc049a/trunk@45 e1591323-3689-4d5a-aa31-d1a7cbdc5706
</commit_message>
<xml_diff>
--- a/www/Manufacturing/artwork/pc049a_lemo_db-manufacturing-artwork-2015-03-04/pc049a_db.xlsx
+++ b/www/Manufacturing/artwork/pc049a_lemo_db-manufacturing-artwork-2015-03-04/pc049a_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="157" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="992" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>TITLE: Bill of Materials</t>
   </si>
@@ -98,7 +98,7 @@
     <t>307-0141</t>
   </si>
   <si>
-    <t>eg. Farnell 2008292 </t>
+    <t>eg. Farnell 2008292</t>
   </si>
   <si>
     <t>TVS_DIODE_ARRAY_SP3010_UDFN-SP3010-04UTG</t>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t> </t>
   </si>
 </sst>
 </file>
@@ -131,6 +128,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -214,40 +212,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="57.5408163265306"/>
     <col collapsed="false" hidden="false" max="2" min="2" style="1" width="76.0204081632653"/>
-    <col collapsed="false" hidden="false" max="1025" min="3" style="0" width="25.515306122449"/>
+    <col collapsed="false" hidden="false" max="5" min="3" style="0" width="25.515306122449"/>
+    <col collapsed="false" hidden="true" max="8" min="6" style="0" width="0"/>
+    <col collapsed="false" hidden="false" max="1025" min="9" style="0" width="25.515306122449"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
@@ -275,7 +283,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="41.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>13</v>
       </c>
@@ -301,7 +309,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="74.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
         <v>18</v>
       </c>
@@ -327,7 +335,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="41.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>21</v>
       </c>
@@ -353,7 +361,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="41.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
         <v>24</v>
       </c>
@@ -379,7 +387,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="41.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
         <v>28</v>
       </c>
@@ -405,36 +413,19 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="41.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C13" s="0" t="n">
+        <f aca="false">SUM(C8:C12)</f>
         <v>113</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="0" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="false" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="false" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>